<commit_message>
Mejoras en el proceso de scraping
</commit_message>
<xml_diff>
--- a/input/input_scraping.xlsx
+++ b/input/input_scraping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\WebScraping\TCGPlayerBot\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663AB027-ACBA-4F39-A296-6043E8FFB6E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD4E17C-D99B-4B61-9472-EA3EE2535903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="690" windowWidth="19185" windowHeight="10710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="21">
   <si>
     <t>set_slug</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t>me04-chaos-rising</t>
+  </si>
+  <si>
+    <t>me05-pitch-black</t>
   </si>
 </sst>
 </file>
@@ -451,7 +454,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -647,6 +650,23 @@
         <v>11</v>
       </c>
     </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>